<commit_message>
feat: expanded catalog to 30 varied products for filter testing
</commit_message>
<xml_diff>
--- a/data/catalog.xlsx
+++ b/data/catalog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1088,9 +1088,963 @@
         <v>C++, Python, Elastic Stack</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TRL-013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>PRODUTO AVANÇADO 13 - Inovação e Pesquisa</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Solução robusta de nível enterprise para Inovação e Pesquisa, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Inovação e Pesquisa</v>
+      </c>
+      <c r="E14" t="str">
+        <v>H2</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Eduardo Rocha</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Zeta</v>
+      </c>
+      <c r="H14" t="str">
+        <v>R$ 4M ARR</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Inovação e Pesquisa</v>
+      </c>
+      <c r="J14" t="str">
+        <v>PME</v>
+      </c>
+      <c r="K14" t="str">
+        <v>H2</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M14" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Inexistência de ferramentas escaláveis de Inovação e Pesquisa no mercado local.</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P14" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TRL-014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>PRODUTO AVANÇADO 14 - S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Solução robusta de nível enterprise para S&amp;M e Inteligência de Mercado, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D15" t="str">
+        <v>S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="E15" t="str">
+        <v>H3</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Fernanda Oliveira</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Eta</v>
+      </c>
+      <c r="H15" t="str">
+        <v>R$ 4M ARR</v>
+      </c>
+      <c r="I15" t="str">
+        <v>S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="J15" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K15" t="str">
+        <v>H3</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M15" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Inexistência de ferramentas escaláveis de S&amp;M e Inteligência de Mercado no mercado local.</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P15" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TRL-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>PRODUTO AVANÇADO 15 - Loss Prevention</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Solução robusta de nível enterprise para Loss Prevention, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Loss Prevention</v>
+      </c>
+      <c r="E16" t="str">
+        <v>H1</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Gustavo Lima</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Theta</v>
+      </c>
+      <c r="H16" t="str">
+        <v>R$ 1M ARR</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Loss Prevention</v>
+      </c>
+      <c r="J16" t="str">
+        <v>PME</v>
+      </c>
+      <c r="K16" t="str">
+        <v>H1</v>
+      </c>
+      <c r="L16" t="str">
+        <v>SaaS Premium</v>
+      </c>
+      <c r="M16" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Inexistência de ferramentas escaláveis de Loss Prevention no mercado local.</v>
+      </c>
+      <c r="O16" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P16" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TRL-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>PRODUTO AVANÇADO 16 - Crédito e Cobrança</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Solução robusta de nível enterprise para Crédito e Cobrança, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Crédito e Cobrança</v>
+      </c>
+      <c r="E17" t="str">
+        <v>H2</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Helena Souza</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Alpha</v>
+      </c>
+      <c r="H17" t="str">
+        <v>R$ 10M ARR</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Crédito e Cobrança</v>
+      </c>
+      <c r="J17" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K17" t="str">
+        <v>H2</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M17" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Inexistência de ferramentas escaláveis de Crédito e Cobrança no mercado local.</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P17" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TRL-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>PRODUTO AVANÇADO 17 - Cotação e Subscrição</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Solução robusta de nível enterprise para Cotação e Subscrição, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Cotação e Subscrição</v>
+      </c>
+      <c r="E18" t="str">
+        <v>H3</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Igor Martins</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Beta</v>
+      </c>
+      <c r="H18" t="str">
+        <v>R$ 10M ARR</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Cotação e Subscrição</v>
+      </c>
+      <c r="J18" t="str">
+        <v>PME</v>
+      </c>
+      <c r="K18" t="str">
+        <v>H3</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M18" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N18" t="str">
+        <v>Inexistência de ferramentas escaláveis de Cotação e Subscrição no mercado local.</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P18" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TRL-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>PRODUTO AVANÇADO 18 - Negócios e Infraestrutura</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Solução robusta de nível enterprise para Negócios e Infraestrutura, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Negócios e Infraestrutura</v>
+      </c>
+      <c r="E19" t="str">
+        <v>H1</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Daniela Lima</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Gamma</v>
+      </c>
+      <c r="H19" t="str">
+        <v>R$ 10M ARR</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Negócios e Infraestrutura</v>
+      </c>
+      <c r="J19" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K19" t="str">
+        <v>H1</v>
+      </c>
+      <c r="L19" t="str">
+        <v>SaaS Premium</v>
+      </c>
+      <c r="M19" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Inexistência de ferramentas escaláveis de Negócios e Infraestrutura no mercado local.</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P19" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TRL-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>PRODUTO AVANÇADO 19 - Capital Markets</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Solução robusta de nível enterprise para Capital Markets, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Capital Markets</v>
+      </c>
+      <c r="E20" t="str">
+        <v>H2</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Carlos Santos</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Delta</v>
+      </c>
+      <c r="H20" t="str">
+        <v>R$ 5M ARR</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Capital Markets</v>
+      </c>
+      <c r="J20" t="str">
+        <v>PME</v>
+      </c>
+      <c r="K20" t="str">
+        <v>H2</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M20" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N20" t="str">
+        <v>Inexistência de ferramentas escaláveis de Capital Markets no mercado local.</v>
+      </c>
+      <c r="O20" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P20" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TRL-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>PRODUTO AVANÇADO 20 - Inovação e Pesquisa</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Solução robusta de nível enterprise para Inovação e Pesquisa, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Inovação e Pesquisa</v>
+      </c>
+      <c r="E21" t="str">
+        <v>H3</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Ana Silva</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Epsilon</v>
+      </c>
+      <c r="H21" t="str">
+        <v>R$ 3M ARR</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Inovação e Pesquisa</v>
+      </c>
+      <c r="J21" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K21" t="str">
+        <v>H3</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M21" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N21" t="str">
+        <v>Inexistência de ferramentas escaláveis de Inovação e Pesquisa no mercado local.</v>
+      </c>
+      <c r="O21" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P21" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TRL-021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>PRODUTO AVANÇADO 21 - S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Solução robusta de nível enterprise para S&amp;M e Inteligência de Mercado, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D22" t="str">
+        <v>S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="E22" t="str">
+        <v>H1</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Bruno Costa</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Zeta</v>
+      </c>
+      <c r="H22" t="str">
+        <v>R$ 9M ARR</v>
+      </c>
+      <c r="I22" t="str">
+        <v>S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="J22" t="str">
+        <v>PME</v>
+      </c>
+      <c r="K22" t="str">
+        <v>H1</v>
+      </c>
+      <c r="L22" t="str">
+        <v>SaaS Premium</v>
+      </c>
+      <c r="M22" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N22" t="str">
+        <v>Inexistência de ferramentas escaláveis de S&amp;M e Inteligência de Mercado no mercado local.</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P22" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TRL-022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>PRODUTO AVANÇADO 22 - Loss Prevention</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Solução robusta de nível enterprise para Loss Prevention, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Loss Prevention</v>
+      </c>
+      <c r="E23" t="str">
+        <v>H2</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Eduardo Rocha</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Eta</v>
+      </c>
+      <c r="H23" t="str">
+        <v>R$ 5M ARR</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Loss Prevention</v>
+      </c>
+      <c r="J23" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K23" t="str">
+        <v>H2</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M23" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Inexistência de ferramentas escaláveis de Loss Prevention no mercado local.</v>
+      </c>
+      <c r="O23" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P23" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TRL-023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>PRODUTO AVANÇADO 23 - Crédito e Cobrança</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Solução robusta de nível enterprise para Crédito e Cobrança, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Crédito e Cobrança</v>
+      </c>
+      <c r="E24" t="str">
+        <v>H3</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Fernanda Oliveira</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Theta</v>
+      </c>
+      <c r="H24" t="str">
+        <v>R$ 6M ARR</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Crédito e Cobrança</v>
+      </c>
+      <c r="J24" t="str">
+        <v>PME</v>
+      </c>
+      <c r="K24" t="str">
+        <v>H3</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M24" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Inexistência de ferramentas escaláveis de Crédito e Cobrança no mercado local.</v>
+      </c>
+      <c r="O24" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P24" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TRL-024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>PRODUTO AVANÇADO 24 - Cotação e Subscrição</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Solução robusta de nível enterprise para Cotação e Subscrição, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Cotação e Subscrição</v>
+      </c>
+      <c r="E25" t="str">
+        <v>H1</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Gustavo Lima</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Alpha</v>
+      </c>
+      <c r="H25" t="str">
+        <v>R$ 4M ARR</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Cotação e Subscrição</v>
+      </c>
+      <c r="J25" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K25" t="str">
+        <v>H1</v>
+      </c>
+      <c r="L25" t="str">
+        <v>SaaS Premium</v>
+      </c>
+      <c r="M25" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Inexistência de ferramentas escaláveis de Cotação e Subscrição no mercado local.</v>
+      </c>
+      <c r="O25" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P25" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TRL-025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>PRODUTO AVANÇADO 25 - Negócios e Infraestrutura</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Solução robusta de nível enterprise para Negócios e Infraestrutura, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Negócios e Infraestrutura</v>
+      </c>
+      <c r="E26" t="str">
+        <v>H2</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Helena Souza</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Beta</v>
+      </c>
+      <c r="H26" t="str">
+        <v>R$ 8M ARR</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Negócios e Infraestrutura</v>
+      </c>
+      <c r="J26" t="str">
+        <v>PME</v>
+      </c>
+      <c r="K26" t="str">
+        <v>H2</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M26" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Inexistência de ferramentas escaláveis de Negócios e Infraestrutura no mercado local.</v>
+      </c>
+      <c r="O26" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P26" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TRL-026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>PRODUTO AVANÇADO 26 - Capital Markets</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Solução robusta de nível enterprise para Capital Markets, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Capital Markets</v>
+      </c>
+      <c r="E27" t="str">
+        <v>H3</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Igor Martins</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Gamma</v>
+      </c>
+      <c r="H27" t="str">
+        <v>R$ 3M ARR</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Capital Markets</v>
+      </c>
+      <c r="J27" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K27" t="str">
+        <v>H3</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M27" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Inexistência de ferramentas escaláveis de Capital Markets no mercado local.</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P27" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TRL-027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>PRODUTO AVANÇADO 27 - Inovação e Pesquisa</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Solução robusta de nível enterprise para Inovação e Pesquisa, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Inovação e Pesquisa</v>
+      </c>
+      <c r="E28" t="str">
+        <v>H1</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Daniela Lima</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Delta</v>
+      </c>
+      <c r="H28" t="str">
+        <v>R$ 7M ARR</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Inovação e Pesquisa</v>
+      </c>
+      <c r="J28" t="str">
+        <v>PME</v>
+      </c>
+      <c r="K28" t="str">
+        <v>H1</v>
+      </c>
+      <c r="L28" t="str">
+        <v>SaaS Premium</v>
+      </c>
+      <c r="M28" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Inexistência de ferramentas escaláveis de Inovação e Pesquisa no mercado local.</v>
+      </c>
+      <c r="O28" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P28" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TRL-028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>PRODUTO AVANÇADO 28 - S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Solução robusta de nível enterprise para S&amp;M e Inteligência de Mercado, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D29" t="str">
+        <v>S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="E29" t="str">
+        <v>H2</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Carlos Santos</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Epsilon</v>
+      </c>
+      <c r="H29" t="str">
+        <v>R$ 3M ARR</v>
+      </c>
+      <c r="I29" t="str">
+        <v>S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="J29" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K29" t="str">
+        <v>H2</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M29" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Inexistência de ferramentas escaláveis de S&amp;M e Inteligência de Mercado no mercado local.</v>
+      </c>
+      <c r="O29" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P29" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TRL-029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>PRODUTO AVANÇADO 29 - Loss Prevention</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Solução robusta de nível enterprise para Loss Prevention, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Loss Prevention</v>
+      </c>
+      <c r="E30" t="str">
+        <v>H3</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Ana Silva</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Zeta</v>
+      </c>
+      <c r="H30" t="str">
+        <v>R$ 8M ARR</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Loss Prevention</v>
+      </c>
+      <c r="J30" t="str">
+        <v>PME</v>
+      </c>
+      <c r="K30" t="str">
+        <v>H3</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Licença Corporativa</v>
+      </c>
+      <c r="M30" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N30" t="str">
+        <v>Inexistência de ferramentas escaláveis de Loss Prevention no mercado local.</v>
+      </c>
+      <c r="O30" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P30" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TRL-030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>PRODUTO AVANÇADO 30 - Crédito e Cobrança</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Solução robusta de nível enterprise para Crédito e Cobrança, otimizada para o ecossistema Trillia.</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Crédito e Cobrança</v>
+      </c>
+      <c r="E31" t="str">
+        <v>H1</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Bruno Costa</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Eta</v>
+      </c>
+      <c r="H31" t="str">
+        <v>R$ 5M ARR</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Crédito e Cobrança</v>
+      </c>
+      <c r="J31" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K31" t="str">
+        <v>H1</v>
+      </c>
+      <c r="L31" t="str">
+        <v>SaaS Premium</v>
+      </c>
+      <c r="M31" t="str">
+        <v>https://trillia.com.br</v>
+      </c>
+      <c r="N31" t="str">
+        <v>Inexistência de ferramentas escaláveis de Crédito e Cobrança no mercado local.</v>
+      </c>
+      <c r="O31" t="str">
+        <v>Automação de workflows, Business intelligence, Segurança de dados</v>
+      </c>
+      <c r="P31" t="str">
+        <v>Microsserviços auto-escaláveis, Lakehouse integration, AI-first architecture</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: Update README and prompt.md with rollback risks and strict definitions
</commit_message>
<xml_diff>
--- a/data/catalog.xlsx
+++ b/data/catalog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:R36"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -451,6 +451,9 @@
       <c r="Q1" t="str">
         <v>tech_stack</v>
       </c>
+      <c r="R1" t="str">
+        <v>owner_email</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -472,7 +475,7 @@
         <v>Ana Silva</v>
       </c>
       <c r="G2" t="str">
-        <v>Alpha</v>
+        <v>SQUAD ALPHA PRIME</v>
       </c>
       <c r="H2" t="str">
         <v>R$ 1.2M ARR</v>
@@ -503,6 +506,9 @@
       </c>
       <c r="Q2" t="str">
         <v>Python, Spark, Power BI, Azure</v>
+      </c>
+      <c r="R2" t="str">
+        <v>ana.silva@trillia.com.br</v>
       </c>
     </row>
     <row r="3">
@@ -525,7 +531,7 @@
         <v>Bruno Costa</v>
       </c>
       <c r="G3" t="str">
-        <v>Alpha</v>
+        <v>SQUAD ALPHA PRIME</v>
       </c>
       <c r="H3" t="str">
         <v>R$ 2.4M ARR</v>
@@ -556,6 +562,9 @@
       </c>
       <c r="Q3" t="str">
         <v>Node.js, MongoDB, React</v>
+      </c>
+      <c r="R3" t="str">
+        <v>bruno.costa@trillia.com.br</v>
       </c>
     </row>
     <row r="4">
@@ -578,7 +587,7 @@
         <v>Carlos Santos</v>
       </c>
       <c r="G4" t="str">
-        <v>Beta</v>
+        <v>SQUAD BETA NEXUS</v>
       </c>
       <c r="H4" t="str">
         <v>R$ 4.8M ARR</v>
@@ -609,6 +618,9 @@
       </c>
       <c r="Q4" t="str">
         <v>Python, TensorFlow, AWS Rekognition</v>
+      </c>
+      <c r="R4" t="str">
+        <v>carlos.santos@trillia.com.br</v>
       </c>
     </row>
     <row r="5">
@@ -631,7 +643,7 @@
         <v>Daniela Lima</v>
       </c>
       <c r="G5" t="str">
-        <v>Beta</v>
+        <v>SQUAD BETA NEXUS</v>
       </c>
       <c r="H5" t="str">
         <v>R$ 7.2M ARR</v>
@@ -662,6 +674,9 @@
       </c>
       <c r="Q5" t="str">
         <v>Go, Redis, Kubernetes</v>
+      </c>
+      <c r="R5" t="str">
+        <v>daniela.lima@trillia.com.br</v>
       </c>
     </row>
     <row r="6">
@@ -684,7 +699,7 @@
         <v>Eduardo Rocha</v>
       </c>
       <c r="G6" t="str">
-        <v>Gamma</v>
+        <v>SQUAD GAMMA CORE</v>
       </c>
       <c r="H6" t="str">
         <v>R$ 3.1M ARR</v>
@@ -715,6 +730,9 @@
       </c>
       <c r="Q6" t="str">
         <v>Java, Spring Boot, PostgreSQL</v>
+      </c>
+      <c r="R6" t="str">
+        <v>eduardo.rocha@trillia.com.br</v>
       </c>
     </row>
     <row r="7">
@@ -737,7 +755,7 @@
         <v>Fernanda Oliveira</v>
       </c>
       <c r="G7" t="str">
-        <v>Gamma</v>
+        <v>SQUAD GAMMA CORE</v>
       </c>
       <c r="H7" t="str">
         <v>R$ 2.5M ARR</v>
@@ -768,6 +786,9 @@
       </c>
       <c r="Q7" t="str">
         <v>PHP (Laravel), MySQL, Twilio</v>
+      </c>
+      <c r="R7" t="str">
+        <v>fernanda.oliveira@trillia.com.br</v>
       </c>
     </row>
     <row r="8">
@@ -790,7 +811,7 @@
         <v>Gustavo Lima</v>
       </c>
       <c r="G8" t="str">
-        <v>Delta</v>
+        <v>SQUAD DELTA FORCE</v>
       </c>
       <c r="H8" t="str">
         <v>R$ 0.8M ARR</v>
@@ -821,6 +842,9 @@
       </c>
       <c r="Q8" t="str">
         <v>C#, .NET Core, SQL Server</v>
+      </c>
+      <c r="R8" t="str">
+        <v>gustavo.lima@trillia.com.br</v>
       </c>
     </row>
     <row r="9">
@@ -843,7 +867,7 @@
         <v>Helena Souza</v>
       </c>
       <c r="G9" t="str">
-        <v>Delta</v>
+        <v>SQUAD DELTA FORCE</v>
       </c>
       <c r="H9" t="str">
         <v>R$ 0.5M ARR</v>
@@ -874,6 +898,9 @@
       </c>
       <c r="Q9" t="str">
         <v>Python, Django, Hyperledger</v>
+      </c>
+      <c r="R9" t="str">
+        <v>helena.souza@trillia.com.br</v>
       </c>
     </row>
     <row r="10">
@@ -896,7 +923,7 @@
         <v>Igor Martins</v>
       </c>
       <c r="G10" t="str">
-        <v>Epsilon</v>
+        <v>SQUAD EPSILON STRAT</v>
       </c>
       <c r="H10" t="str">
         <v>R$ 1.8M ARR</v>
@@ -927,6 +954,9 @@
       </c>
       <c r="Q10" t="str">
         <v>Rust, WebAssembly, ClickHouse</v>
+      </c>
+      <c r="R10" t="str">
+        <v>igor.martins@trillia.com.br</v>
       </c>
     </row>
     <row r="11">
@@ -949,7 +979,7 @@
         <v>Helena Souza</v>
       </c>
       <c r="G11" t="str">
-        <v>Epsilon</v>
+        <v>SQUAD EPSILON STRAT</v>
       </c>
       <c r="H11" t="str">
         <v>R$ 0 ARR</v>
@@ -980,6 +1010,9 @@
       </c>
       <c r="Q11" t="str">
         <v>Q#, Python, Azure Quantum</v>
+      </c>
+      <c r="R11" t="str">
+        <v>helena.souza@trillia.com.br</v>
       </c>
     </row>
     <row r="12">
@@ -1002,7 +1035,7 @@
         <v>Igor Martins</v>
       </c>
       <c r="G12" t="str">
-        <v>Delta</v>
+        <v>SQUAD DELTA FORCE</v>
       </c>
       <c r="H12" t="str">
         <v>R$ 0.3M ARR</v>
@@ -1033,6 +1066,9 @@
       </c>
       <c r="Q12" t="str">
         <v>Solidity, Ethereum, Infura</v>
+      </c>
+      <c r="R12" t="str">
+        <v>igor.martins@trillia.com.br</v>
       </c>
     </row>
     <row r="13">
@@ -1055,7 +1091,7 @@
         <v>Carlos Santos</v>
       </c>
       <c r="G13" t="str">
-        <v>Beta</v>
+        <v>SQUAD BETA NEXUS</v>
       </c>
       <c r="H13" t="str">
         <v>R$ 5.5M ARR</v>
@@ -1086,6 +1122,9 @@
       </c>
       <c r="Q13" t="str">
         <v>C++, Python, Elastic Stack</v>
+      </c>
+      <c r="R13" t="str">
+        <v>carlos.santos@trillia.com.br</v>
       </c>
     </row>
     <row r="14">
@@ -1108,7 +1147,7 @@
         <v>Eduardo Rocha</v>
       </c>
       <c r="G14" t="str">
-        <v>Zeta</v>
+        <v>SQUAD ZETA VISION</v>
       </c>
       <c r="H14" t="str">
         <v>R$ 4M ARR</v>
@@ -1139,6 +1178,9 @@
       </c>
       <c r="Q14" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R14" t="str">
+        <v>eduardo.rocha@trillia.com.br</v>
       </c>
     </row>
     <row r="15">
@@ -1161,7 +1203,7 @@
         <v>Fernanda Oliveira</v>
       </c>
       <c r="G15" t="str">
-        <v>Eta</v>
+        <v>SQUAD ETA SOLUTIONS</v>
       </c>
       <c r="H15" t="str">
         <v>R$ 4M ARR</v>
@@ -1192,6 +1234,9 @@
       </c>
       <c r="Q15" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R15" t="str">
+        <v>fernanda.oliveira@trillia.com.br</v>
       </c>
     </row>
     <row r="16">
@@ -1214,7 +1259,7 @@
         <v>Gustavo Lima</v>
       </c>
       <c r="G16" t="str">
-        <v>Theta</v>
+        <v>SQUAD THETA LABS</v>
       </c>
       <c r="H16" t="str">
         <v>R$ 1M ARR</v>
@@ -1245,6 +1290,9 @@
       </c>
       <c r="Q16" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R16" t="str">
+        <v>gustavo.lima@trillia.com.br</v>
       </c>
     </row>
     <row r="17">
@@ -1267,7 +1315,7 @@
         <v>Helena Souza</v>
       </c>
       <c r="G17" t="str">
-        <v>Alpha</v>
+        <v>SQUAD ALPHA PRIME</v>
       </c>
       <c r="H17" t="str">
         <v>R$ 10M ARR</v>
@@ -1298,6 +1346,9 @@
       </c>
       <c r="Q17" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R17" t="str">
+        <v>helena.souza@trillia.com.br</v>
       </c>
     </row>
     <row r="18">
@@ -1320,7 +1371,7 @@
         <v>Igor Martins</v>
       </c>
       <c r="G18" t="str">
-        <v>Beta</v>
+        <v>SQUAD BETA NEXUS</v>
       </c>
       <c r="H18" t="str">
         <v>R$ 10M ARR</v>
@@ -1351,6 +1402,9 @@
       </c>
       <c r="Q18" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R18" t="str">
+        <v>igor.martins@trillia.com.br</v>
       </c>
     </row>
     <row r="19">
@@ -1373,7 +1427,7 @@
         <v>Daniela Lima</v>
       </c>
       <c r="G19" t="str">
-        <v>Gamma</v>
+        <v>SQUAD GAMMA CORE</v>
       </c>
       <c r="H19" t="str">
         <v>R$ 10M ARR</v>
@@ -1404,6 +1458,9 @@
       </c>
       <c r="Q19" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R19" t="str">
+        <v>daniela.lima@trillia.com.br</v>
       </c>
     </row>
     <row r="20">
@@ -1426,7 +1483,7 @@
         <v>Carlos Santos</v>
       </c>
       <c r="G20" t="str">
-        <v>Delta</v>
+        <v>SQUAD DELTA FORCE</v>
       </c>
       <c r="H20" t="str">
         <v>R$ 5M ARR</v>
@@ -1457,6 +1514,9 @@
       </c>
       <c r="Q20" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R20" t="str">
+        <v>carlos.santos@trillia.com.br</v>
       </c>
     </row>
     <row r="21">
@@ -1479,7 +1539,7 @@
         <v>Ana Silva</v>
       </c>
       <c r="G21" t="str">
-        <v>Epsilon</v>
+        <v>SQUAD EPSILON STRAT</v>
       </c>
       <c r="H21" t="str">
         <v>R$ 3M ARR</v>
@@ -1510,6 +1570,9 @@
       </c>
       <c r="Q21" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R21" t="str">
+        <v>ana.silva@trillia.com.br</v>
       </c>
     </row>
     <row r="22">
@@ -1532,7 +1595,7 @@
         <v>Bruno Costa</v>
       </c>
       <c r="G22" t="str">
-        <v>Zeta</v>
+        <v>SQUAD ZETA VISION</v>
       </c>
       <c r="H22" t="str">
         <v>R$ 9M ARR</v>
@@ -1563,6 +1626,9 @@
       </c>
       <c r="Q22" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R22" t="str">
+        <v>bruno.costa@trillia.com.br</v>
       </c>
     </row>
     <row r="23">
@@ -1585,7 +1651,7 @@
         <v>Eduardo Rocha</v>
       </c>
       <c r="G23" t="str">
-        <v>Eta</v>
+        <v>SQUAD ETA SOLUTIONS</v>
       </c>
       <c r="H23" t="str">
         <v>R$ 5M ARR</v>
@@ -1616,6 +1682,9 @@
       </c>
       <c r="Q23" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R23" t="str">
+        <v>eduardo.rocha@trillia.com.br</v>
       </c>
     </row>
     <row r="24">
@@ -1638,7 +1707,7 @@
         <v>Fernanda Oliveira</v>
       </c>
       <c r="G24" t="str">
-        <v>Theta</v>
+        <v>SQUAD THETA LABS</v>
       </c>
       <c r="H24" t="str">
         <v>R$ 6M ARR</v>
@@ -1669,6 +1738,9 @@
       </c>
       <c r="Q24" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R24" t="str">
+        <v>fernanda.oliveira@trillia.com.br</v>
       </c>
     </row>
     <row r="25">
@@ -1691,7 +1763,7 @@
         <v>Gustavo Lima</v>
       </c>
       <c r="G25" t="str">
-        <v>Alpha</v>
+        <v>SQUAD ALPHA PRIME</v>
       </c>
       <c r="H25" t="str">
         <v>R$ 4M ARR</v>
@@ -1722,6 +1794,9 @@
       </c>
       <c r="Q25" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R25" t="str">
+        <v>gustavo.lima@trillia.com.br</v>
       </c>
     </row>
     <row r="26">
@@ -1744,7 +1819,7 @@
         <v>Helena Souza</v>
       </c>
       <c r="G26" t="str">
-        <v>Beta</v>
+        <v>SQUAD BETA NEXUS</v>
       </c>
       <c r="H26" t="str">
         <v>R$ 8M ARR</v>
@@ -1775,6 +1850,9 @@
       </c>
       <c r="Q26" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R26" t="str">
+        <v>helena.souza@trillia.com.br</v>
       </c>
     </row>
     <row r="27">
@@ -1797,7 +1875,7 @@
         <v>Igor Martins</v>
       </c>
       <c r="G27" t="str">
-        <v>Gamma</v>
+        <v>SQUAD GAMMA CORE</v>
       </c>
       <c r="H27" t="str">
         <v>R$ 3M ARR</v>
@@ -1828,6 +1906,9 @@
       </c>
       <c r="Q27" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R27" t="str">
+        <v>igor.martins@trillia.com.br</v>
       </c>
     </row>
     <row r="28">
@@ -1850,7 +1931,7 @@
         <v>Daniela Lima</v>
       </c>
       <c r="G28" t="str">
-        <v>Delta</v>
+        <v>SQUAD DELTA FORCE</v>
       </c>
       <c r="H28" t="str">
         <v>R$ 7M ARR</v>
@@ -1881,6 +1962,9 @@
       </c>
       <c r="Q28" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R28" t="str">
+        <v>daniela.lima@trillia.com.br</v>
       </c>
     </row>
     <row r="29">
@@ -1903,7 +1987,7 @@
         <v>Carlos Santos</v>
       </c>
       <c r="G29" t="str">
-        <v>Epsilon</v>
+        <v>SQUAD EPSILON STRAT</v>
       </c>
       <c r="H29" t="str">
         <v>R$ 3M ARR</v>
@@ -1934,6 +2018,9 @@
       </c>
       <c r="Q29" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R29" t="str">
+        <v>carlos.santos@trillia.com.br</v>
       </c>
     </row>
     <row r="30">
@@ -1956,7 +2043,7 @@
         <v>Ana Silva</v>
       </c>
       <c r="G30" t="str">
-        <v>Zeta</v>
+        <v>SQUAD ZETA VISION</v>
       </c>
       <c r="H30" t="str">
         <v>R$ 8M ARR</v>
@@ -1987,6 +2074,9 @@
       </c>
       <c r="Q30" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
+      </c>
+      <c r="R30" t="str">
+        <v>ana.silva@trillia.com.br</v>
       </c>
     </row>
     <row r="31">
@@ -2009,7 +2099,7 @@
         <v>Bruno Costa</v>
       </c>
       <c r="G31" t="str">
-        <v>Eta</v>
+        <v>SQUAD ETA SOLUTIONS</v>
       </c>
       <c r="H31" t="str">
         <v>R$ 5M ARR</v>
@@ -2041,10 +2131,293 @@
       <c r="Q31" t="str">
         <v>TypeScript, Docker, AWS, Snowflake</v>
       </c>
+      <c r="R31" t="str">
+        <v>bruno.costa@trillia.com.br</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TRL-031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>REAL-TIME LIQUIDITY MONITOR</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Monitoramento contínuo de liquidez para ativos de Capital Markets.</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Capital Markets</v>
+      </c>
+      <c r="E32" t="str">
+        <v>H1</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Fernanda Oliveira</v>
+      </c>
+      <c r="G32" t="str">
+        <v>SQUAD DELTA FORCE</v>
+      </c>
+      <c r="H32" t="str">
+        <v>R$ 800k ARR</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Capital Markets</v>
+      </c>
+      <c r="J32" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K32" t="str">
+        <v>H1</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Mensal</v>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
+      <c r="N32" t="str">
+        <v>Gargalos de liquidez não detectados.</v>
+      </c>
+      <c r="O32" t="str">
+        <v>Monitoramento, Alertas, Dashboard</v>
+      </c>
+      <c r="P32" t="str">
+        <v>Streaming de Dados, In-memory DB</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>C#, Kafka, Redis</v>
+      </c>
+      <c r="R32" t="str">
+        <v>fernanda.oliveira@trillia.com.br</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TRL-032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>ESG SCORING ENGINE</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Motor de score baseado em critérios ESG para portfólios de investimento.</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Inovação e Pesquisa</v>
+      </c>
+      <c r="E33" t="str">
+        <v>H2</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Gabriel Silva</v>
+      </c>
+      <c r="G33" t="str">
+        <v>SQUAD DEEP DIVE AI</v>
+      </c>
+      <c r="H33" t="str">
+        <v>R$ 500k ARR</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Inovação e Pesquisa</v>
+      </c>
+      <c r="J33" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K33" t="str">
+        <v>H2</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Anual</v>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v>Dificuldade em quantificar impacto ESG.</v>
+      </c>
+      <c r="O33" t="str">
+        <v>Rating, Compliance, Relatórios</v>
+      </c>
+      <c r="P33" t="str">
+        <v>NLP para relatórios, Modelos Estatísticos</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>Python, PyTorch, MongoDB</v>
+      </c>
+      <c r="R33" t="str">
+        <v>gabriel.silva@trillia.com.br</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TRL-033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>PREDICTIVE CHURN AI</v>
+      </c>
+      <c r="C34" t="str">
+        <v>IA para predizer cancelamentos de clientes em tempo real.</v>
+      </c>
+      <c r="D34" t="str">
+        <v>S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="E34" t="str">
+        <v>H1</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Ana Silva</v>
+      </c>
+      <c r="G34" t="str">
+        <v>SQUAD ALPHA PRIME</v>
+      </c>
+      <c r="H34" t="str">
+        <v>R$ 1.5M ARR</v>
+      </c>
+      <c r="I34" t="str">
+        <v>S&amp;M e Inteligência de Mercado</v>
+      </c>
+      <c r="J34" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K34" t="str">
+        <v>H1</v>
+      </c>
+      <c r="L34" t="str">
+        <v>SaaS</v>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v>Alta taxa de cancelamento sem aviso prévio.</v>
+      </c>
+      <c r="O34" t="str">
+        <v>Retenção, Scoring de Churn</v>
+      </c>
+      <c r="P34" t="str">
+        <v>Random Forests, XGBoost</v>
+      </c>
+      <c r="Q34" t="str">
+        <v>Python, Scikit-learn, Snowflake</v>
+      </c>
+      <c r="R34" t="str">
+        <v>ana.silva@trillia.com.br</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TRL-034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>AUTO-SETTLEMENT NODE</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Liquidação automática de ativos via redes distribuídas.</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Negócios e Infraestrutura</v>
+      </c>
+      <c r="E35" t="str">
+        <v>H3</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Lucas Mendes</v>
+      </c>
+      <c r="G35" t="str">
+        <v>SQUAD QUANTUM COMPUTING</v>
+      </c>
+      <c r="H35" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Negócios e Infraestrutura</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Web3</v>
+      </c>
+      <c r="K35" t="str">
+        <v>H3</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Transacional</v>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v>Lentidão em processos de liquidez tradicionais.</v>
+      </c>
+      <c r="O35" t="str">
+        <v>Settlement, Trustless Transactions</v>
+      </c>
+      <c r="P35" t="str">
+        <v>Smart Contracts, Blockchain Layer 2</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>Solidity, Rust, Ethereum</v>
+      </c>
+      <c r="R35" t="str">
+        <v>lucas.mendes@trillia.com.br</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TRL-035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>DYNAMIC PRICING BOT</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Ajuste automático de preços para cotações complexas.</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Cotação e Subscrição</v>
+      </c>
+      <c r="E36" t="str">
+        <v>H2</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Roberto Mendes</v>
+      </c>
+      <c r="G36" t="str">
+        <v>SQUAD GAMMA CORE</v>
+      </c>
+      <c r="H36" t="str">
+        <v>R$ 1.2M ARR</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Cotação e Subscrição</v>
+      </c>
+      <c r="J36" t="str">
+        <v>B2B</v>
+      </c>
+      <c r="K36" t="str">
+        <v>H2</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Percentual de Margem</v>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v>Margens baixas por precificação estática.</v>
+      </c>
+      <c r="O36" t="str">
+        <v>Otimização de Preço, Cotação Automática</v>
+      </c>
+      <c r="P36" t="str">
+        <v>Algoritmos Genéticos, Simulação Monte Carlo</v>
+      </c>
+      <c r="Q36" t="str">
+        <v>Node.js, C++</v>
+      </c>
+      <c r="R36" t="str">
+        <v>roberto.mendes@trillia.com.br</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>